<commit_message>
feat: rework project management and project-scoped RBAC
</commit_message>
<xml_diff>
--- a/projects/mini-rally/07_Testing Plan/02_test_phase_5_6/PHASE_0_6_AUDIT_TRACKER.xlsx
+++ b/projects/mini-rally/07_Testing Plan/02_test_phase_5_6/PHASE_0_6_AUDIT_TRACKER.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1b214e27a60a44f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Guide" sheetId="2" r:id="R6171b57647fa4c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Plan" sheetId="3" r:id="R876163687d2c46b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carryover P0-4" sheetId="4" r:id="Rac4787d30275477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 5 Scenarios" sheetId="5" r:id="Rf7fbeff35e6c4085"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6 Scenarios" sheetId="6" r:id="Rfbc672800b1345a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="7" r:id="R67134e609a4246ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rbb647fea2d1f44d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Guide" sheetId="2" r:id="R7c66b23422064669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution Plan" sheetId="3" r:id="R11efd530b46f494f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carryover P0-4" sheetId="4" r:id="R148530cc6d21441d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 5 Scenarios" sheetId="5" r:id="R074970e2ba0d482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 6 Scenarios" sheetId="6" r:id="R0eb63fb4a75046e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run Log" sheetId="7" r:id="Rcc8e87e4601e44ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Current Access Baseline" sheetId="8" r:id="R0e6053c811784415"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +24,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -57,8 +58,25 @@
       <x:color rgb="FF173F73"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF455A70"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF25364A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF2E6B3A"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -90,8 +108,23 @@
         <x:fgColor rgb="FFFFF8E7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF173F73"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2B62A8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="10">
+  <x:borders count="13">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -183,11 +216,32 @@
         <x:color rgb="FFC8D5E5"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFDCE5EF"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFDCE5EF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFDCE5EF"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFDCE5EF"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8D5E5"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="93">
+  <x:cellXfs count="121">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -403,6 +457,68 @@
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -629,7 +745,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Phase 0-4 carryover plus Phase 5-6 deployed-product acceptance. Updated 2026-08-06.</x:v>
+        <x:v>Phase 0-6 deployed-product audit. Fail/Partial re-test completed 2026-08-09; current Project access baseline added 2026-08-10.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -658,8 +774,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="B5" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A5)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A5)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A5)</x:f>
-        <x:v>67</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D5" s="77" t="str">
         <x:v>Carryover P0-4</x:v>
@@ -673,8 +788,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="B6" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A6)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A6)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A6)</x:f>
-        <x:v>33</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="D6" s="77" t="str">
         <x:v>Phase 5 scenarios</x:v>
@@ -688,8 +802,7 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="B7" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A7)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A7)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A7)</x:f>
-        <x:v>24</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D7" s="77" t="str">
         <x:v>Phase 6 scenarios</x:v>
@@ -703,7 +816,6 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B8" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A8)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A8)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A8)</x:f>
         <x:v>14</x:v>
       </x:c>
       <x:c r="D8" s="77" t="str">
@@ -719,7 +831,6 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="B9" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A9)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A9)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A9)</x:f>
         <x:v>41</x:v>
       </x:c>
       <x:c r="D9" s="77"/>
@@ -730,7 +841,6 @@
         <x:v>Future Backlog</x:v>
       </x:c>
       <x:c r="B10" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A10)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A10)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A10)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D10" s="77" t="str">
@@ -746,7 +856,6 @@
         <x:v>Not Required</x:v>
       </x:c>
       <x:c r="B11" s="77" t="n">
-        <x:f>COUNTIF('Carryover P0-4'!$L$5:$L$65,A11)+COUNTIF('Phase 5 Scenarios'!$L$5:$L$82,A11)+COUNTIF('Phase 6 Scenarios'!$L$5:$L$57,A11)</x:f>
         <x:v>4</x:v>
       </x:c>
     </x:row>
@@ -788,10 +897,10 @@
         <x:v>Test accounts</x:v>
       </x:c>
       <x:c r="C15" s="83" t="str">
-        <x:v>Project Admin and Project Member sessions are required</x:v>
+        <x:v>Workspace Admin plus Project-scoped Admin, Editor, Viewer, and No Access sessions are required</x:v>
       </x:c>
       <x:c r="D15" s="83" t="str">
-        <x:v>Blocks RBAC and denied-route proof</x:v>
+        <x:v>Blocks current access-level and denied-route proof</x:v>
       </x:c>
       <x:c r="E15" s="83"/>
       <x:c r="F15" s="83"/>
@@ -1084,13 +1193,13 @@
         <x:v>Navigation and RBAC</x:v>
       </x:c>
       <x:c r="D7" s="83" t="str">
-        <x:v>Three test roles</x:v>
+        <x:v>WA plus Admin, Editor, Viewer, and No Access profiles</x:v>
       </x:c>
       <x:c r="E7" s="83" t="str">
         <x:v>Portfolio routes, scope and action gates</x:v>
       </x:c>
       <x:c r="F7" s="83" t="str">
-        <x:v>Role matrix confirmed</x:v>
+        <x:v>Current access baseline confirmed</x:v>
       </x:c>
       <x:c r="G7" s="83" t="str">
         <x:v>BA/User</x:v>
@@ -1317,7 +1426,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>61 unresolved, blocked, deferred or Future Backlog rows carried from DEVINT Phase 0-4 audit.</x:v>
+        <x:v>Historical Phase 0-4 carryover. Current Project authorization is defined in Current Access Baseline; former global Project role wording is retained only as execution history.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -1466,7 +1575,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E6" s="38" t="str">
-        <x:v>Portfolio menu behavior</x:v>
+        <x:v>Portfolio menu behavior — C2 reconciled</x:v>
       </x:c>
       <x:c r="F6" s="38" t="str">
         <x:v>DevInt truy cập được và không có lỗi tải trang nghiêm trọng.
@@ -1476,18 +1585,13 @@
         <x:v>Dùng dữ liệu test riêng trong Project TEST. Nếu chưa có dữ liệu bắt buộc, ghi Blocked và nêu rõ dữ liệu còn thiếu.</x:v>
       </x:c>
       <x:c r="H6" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở global header/navigation; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình Global navigation, kiểm tra chức năng "Portfolio menu behavior" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: DevInt renders Portfolio as a direct link to /portfolio and has no Release Planning dropdown item..
-8. Kiểm tra hướng sửa đã chốt: Convert Portfolio to a dropdown and add Release Planning as a Phase 5 entry marked Coming Soon until Phase 5. Do not expose Release create/edit there. Reconcile mockup and navigation documents after the full audit..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open DevInt and inspect Portfolio navigation.
+2. Verify Portfolio Items, Capacity Planning and Release Tracking are available.
+3. Confirm Release Planning is not an active entry and remains Future Backlog.
+4. Record the result without treating the absent Release Planning entry as a defect.</x:v>
       </x:c>
       <x:c r="I6" s="38" t="str">
-        <x:v>Portfolio is a dropdown containing Release Planning. Release Planning is a Phase 5 placeholder and is not a second Release management source in Phase 0–4.</x:v>
+        <x:v>Portfolio dropdown contains Portfolio Items, Capacity Planning and Release Tracking. Release Planning remains Future Backlog and is not an active navigation item.</x:v>
       </x:c>
       <x:c r="J6" s="38" t="str">
         <x:v>P0-SHELL-01</x:v>
@@ -1496,25 +1600,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L6" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M6" s="51" t="str">
-        <x:v>Portfolio is a dropdown with Portfolio Items, Capacity Planning and Release Tracking. Historical Release Planning is absent; BA trace alignment is still needed.</x:v>
+        <x:v>Pass / Not a Defect. DevInt matches the C2-confirmed Portfolio menu; the historical Release Planning expectation was stale.</x:v>
       </x:c>
       <x:c r="N6" s="51" t="str">
         <x:v>evidence/retest_2026-07-24/P0-SHELL-01-dev.png; evidence/retest_2026-07-24/P0-SHELL-01-mock.png</x:v>
       </x:c>
       <x:c r="O6" s="51" t="str">
-        <x:v>Align the historical Release Planning expectation with the approved Portfolio menu.</x:v>
+        <x:v>Closed by BA decision C2. No DEV fix required for this gap.</x:v>
       </x:c>
       <x:c r="P6" s="51" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="Q6" s="51" t="str">
-        <x:v>Fix Direction Approved</x:v>
-      </x:c>
-      <x:c r="R6" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Confirmed C2 — Closed / Not a Defect</x:v>
+      </x:c>
+      <x:c r="R6" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2228,22 +2332,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M18" s="51" t="str">
-        <x:v>Backlog search clearing is not reliable: P56-AUDIT Carryover Story remained in the search box/list until reload.</x:v>
+        <x:v>Re-test 2026-08-09: Search filters to one matching row, but clearing the search field leaves the filtered row and 1–1 of 1 until reload.</x:v>
       </x:c>
       <x:c r="N18" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P1-BL-01-list-states.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O18" s="51" t="str">
-        <x:v>Fix normal clear behavior without reload.</x:v>
+        <x:v>DEV: clearing Backlog search must restore the full scoped list without reload.</x:v>
       </x:c>
       <x:c r="P18" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q18" s="51" t="str">
-        <x:v>Fix Direction Approved</x:v>
-      </x:c>
-      <x:c r="R18" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R18" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2290,25 +2394,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L19" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M19" s="51" t="str">
-        <x:v>Priority filter offers values, but selecting None retained both the Defect and Story. Story must not be treated as Priority None.</x:v>
+        <x:v>Re-test 2026-08-09: Priority=None returned only DE-1; Story rows were excluded.</x:v>
       </x:c>
       <x:c r="N19" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P1-BL-01-list-states.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O19" s="51" t="str">
-        <x:v>Restrict Priority filtering to Defects; Stories remain dash.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P19" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q19" s="51" t="str">
-        <x:v>Fix Direction Approved</x:v>
-      </x:c>
-      <x:c r="R19" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R19" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -2566,7 +2670,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E24" s="38" t="str">
-        <x:v>Team selector contains invalid project team</x:v>
+        <x:v>Team optional and Project/Team scope — C1 reconciled</x:v>
       </x:c>
       <x:c r="F24" s="38" t="str">
         <x:v>DevInt truy cập được và không có lỗi tải trang nghiêm trọng.
@@ -2577,18 +2681,13 @@
         <x:v>Project TEST; một Team có member và một Team không có member; Team Lead để trống khi case yêu cầu.</x:v>
       </x:c>
       <x:c r="H24" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở Work Item Create; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình Work Item Create, kiểm tra chức năng "Team selector contains invalid project team" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: In DevInt NXP / All Teams, the modal listed No team and Team Alpha. Selecting Team Alpha and submitting returned Team is not linked to this project..
-8. Kiểm tra hướng sửa đã chốt: Make the Project dropdown drive the required Team options. Remove No team. List only active Teams linked to the selected Project; if the Project has no valid Team, disable create and show a clear Team validation/empty state..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open Work Item Quick Create.
+2. Select a Project and leave Team as No team; confirm the item belongs to the Project backlog.
+3. Select a Team; confirm only Teams linked to the Project are allowed.
+4. Verify the same rule in Work Item Detail.</x:v>
       </x:c>
       <x:c r="I24" s="38" t="str">
-        <x:v>Team is required. Team options in Work Item create are filtered to Teams linked to the selected/current Project; No team and invalid Team/Project combinations cannot be selected.</x:v>
+        <x:v>Project is required. Team is optional: No team creates the Work Item in the Project backlog; a selected Team must be linked to the Project.</x:v>
       </x:c>
       <x:c r="J24" s="38" t="str">
         <x:v>P1-CREATE-01</x:v>
@@ -2597,25 +2696,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L24" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M24" s="51" t="str">
-        <x:v>Team selector exposes No team and Pegasus. This matches the newer BA Project-backlog rule but conflicts with historical required-Team wording.</x:v>
+        <x:v>Pass / Not a Defect. No team is valid under the C1-confirmed Project backlog rule.</x:v>
       </x:c>
       <x:c r="N24" s="51" t="str">
         <x:v>evidence/retest_2026-07-24/P1-CREATE-01-quick-create.png</x:v>
       </x:c>
       <x:c r="O24" s="51" t="str">
-        <x:v>Update SRS/mockup trace to the approved no-team Project backlog rule.</x:v>
+        <x:v>Closed by BA decision C1. Invalid cross-Project Team options remain prohibited.</x:v>
       </x:c>
       <x:c r="P24" s="51" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="Q24" s="51" t="str">
-        <x:v>Fix Direction Approved</x:v>
-      </x:c>
-      <x:c r="R24" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Confirmed C1 — Closed / Not a Defect</x:v>
+      </x:c>
+      <x:c r="R24" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2654,7 +2753,7 @@
 9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
       </x:c>
       <x:c r="I25" s="38" t="str">
-        <x:v>Owner defaults to the authenticated/current user, lists users valid for the selected Project/Team, and also allows an explicit Unassigned choice.</x:v>
+        <x:v>Owner defaults to the authenticated/current user, includes an explicit Unassigned option, and lists only users valid for the selected Project/Team.</x:v>
       </x:c>
       <x:c r="J25" s="38" t="str">
         <x:v>P1-CREATE-01</x:v>
@@ -2666,22 +2765,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M25" s="51" t="str">
-        <x:v>Owner defaults to Unassigned. After Hieu was added to Pegasus, Settings &gt; Teams showed Anh and Hieu, but the US-1 Owner dropdown still showed only No Entry and Anh. Owner membership options did not refresh from current Team membership.</x:v>
+        <x:v>Re-test 2026-08-09: quick create still defaults Owner to Unassigned. Owner choices show No Entry and Anh only; current user is not selectable.</x:v>
       </x:c>
       <x:c r="N25" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O25" s="51" t="str">
-        <x:v>Keep the approved default rule. Source every Owner selector from current Project/Team membership and invalidate stale membership options after a member is added or removed.</x:v>
+        <x:v>DEV: align Owner default and membership-scoped options with the approved rule.</x:v>
       </x:c>
       <x:c r="P25" s="51" t="str">
-        <x:v>BA + Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q25" s="51" t="str">
-        <x:v>Bug confirmed; membership sync required</x:v>
+        <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R25" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2999,7 +3098,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="E31" s="38" t="str">
-        <x:v>Required Team and No team option</x:v>
+        <x:v>Optional Team and Project backlog — C1 reconciled</x:v>
       </x:c>
       <x:c r="F31" s="38" t="str">
         <x:v>DevInt truy cập được và không có lỗi tải trang nghiêm trọng.
@@ -3009,18 +3108,13 @@
         <x:v>Project TEST; một Team có member và một Team không có member; Team Lead để trống khi case yêu cầu.</x:v>
       </x:c>
       <x:c r="H31" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở Backlog or Iteration Status &gt; Work Item Detail; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình Work Item Detail, kiểm tra chức năng "Required Team and No team option" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: DevInt US-7 Team dropdown includes No team and Team Alpha while Project is not displayed..
-8. Kiểm tra hướng sửa đã chốt: Remove No team from Work Item Detail and filter Team options by Project. Apply the same required linked-Team rule in Quick Create and Detail..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open an existing Work Item Detail.
+2. Set Team to No team and verify it remains in the Project backlog.
+3. Select a Team and verify it is linked to the Work Item Project.
+4. Confirm Quick Create and Detail use the same rule.</x:v>
       </x:c>
       <x:c r="I31" s="38" t="str">
-        <x:v>Team remains required for a Work Item and must be linked to the selected Project; No team is not an allowed value.</x:v>
+        <x:v>Team is optional. No team is valid and keeps the Work Item in the Project backlog; any selected Team must be linked to the Project.</x:v>
       </x:c>
       <x:c r="J31" s="38" t="str">
         <x:v>P1-WID-01</x:v>
@@ -3029,25 +3123,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L31" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M31" s="51" t="str">
-        <x:v>Quick Create still offers No team; it matches newer BA decision but conflicts with historical SRS wording.</x:v>
+        <x:v>Pass / Not a Defect. C1 confirms No team is valid in both Quick Create and Detail.</x:v>
       </x:c>
       <x:c r="N31" s="51" t="str">
         <x:v>evidence/retest_2026-07-24/P1-WID-01-US-13-detail.png</x:v>
       </x:c>
       <x:c r="O31" s="51" t="str">
-        <x:v>Update SRS/mockup trace before formal Pass.</x:v>
+        <x:v>Closed by BA decision C1.</x:v>
       </x:c>
       <x:c r="P31" s="51" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="Q31" s="51" t="str">
-        <x:v>Fix Direction Approved</x:v>
-      </x:c>
-      <x:c r="R31" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Confirmed C1 — Closed / Not a Defect</x:v>
+      </x:c>
+      <x:c r="R31" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -3489,7 +3583,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="E39" s="38" t="str">
-        <x:v>Missing Project and Task Estimate columns</x:v>
+        <x:v>Missing Task Estimate column — C9 narrowed</x:v>
       </x:c>
       <x:c r="F39" s="38" t="str">
         <x:v>DevInt truy cập được và không có lỗi tải trang nghiêm trọng.
@@ -3499,18 +3593,12 @@
         <x:v>Project TEST; một Iteration active và một Iteration completed; Work Item/Task có thể nhận biết bằng prefix P56-AUDIT.</x:v>
       </x:c>
       <x:c r="H39" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở Timeboxes &gt; Iterations list; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình Timeboxes &gt; Iterations list, kiểm tra chức năng "Missing Project and Task Estimate columns" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: DevInt list shows ID, Name, Theme, Start Date, End Date, Planned Velocity and State only. Project and Task Estimate are absent..
-8. Kiểm tra hướng sửa đã chốt: Add the Project and Task Estimate columns to the Iterations list using the existing list contract..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open Timeboxes &gt; Iterations in a single-Project scope.
+2. Verify the list omits Project column/search/sort.
+3. Verify Task Estimate is present and reflects the Iteration Task total.</x:v>
       </x:c>
       <x:c r="I39" s="38" t="str">
-        <x:v>Iterations list shows Name, Theme, Start Date, End Date, Project, Planned Velocity, Task Estimate and State (P2-IT-FR-005).</x:v>
+        <x:v>Iteration list shows ID, Name, Theme, Start Date, End Date, Planned Velocity, Task Estimate and State. Project column/search/sort is omitted in single-Project scope.</x:v>
       </x:c>
       <x:c r="J39" s="38" t="str">
         <x:v>P2-IT-01</x:v>
@@ -3519,25 +3607,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L39" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M39" s="51" t="str">
-        <x:v>Iteration list has ID, Name, Theme, Start Date, End Date, Planned Velocity and State; Project and Task Estimate columns are absent.</x:v>
+        <x:v>Re-test 2026-08-09: Iteration list now includes Task Estimate and correctly omits Project in single-Project scope.</x:v>
       </x:c>
       <x:c r="N39" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P2-IT-01-timeboxes.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/timeboxes</x:v>
       </x:c>
       <x:c r="O39" s="51" t="str">
-        <x:v>Add the approved Project and Task Estimate columns.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P39" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q39" s="51" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="R39" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R39" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -3554,7 +3642,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="E40" s="38" t="str">
-        <x:v>Missing Type column</x:v>
+        <x:v>Type column not required — C3 reconciled</x:v>
       </x:c>
       <x:c r="F40" s="38" t="str">
         <x:v>DevInt truy cập được và không có lỗi tải trang nghiêm trọng.
@@ -3564,18 +3652,12 @@
         <x:v>Project TEST; một Iteration active và một Iteration completed; Work Item/Task có thể nhận biết bằng prefix P56-AUDIT.</x:v>
       </x:c>
       <x:c r="H40" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở Iteration Status list; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình Iteration Status list, kiểm tra chức năng "Missing Type column" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: DevInt list has no Type column; it also adds Feature, Blocked Reason, Tasks, Actual, Defect Status, Milestones and Dev Owner beyond the contract..
-8. Kiểm tra hướng sửa đã chốt: Add the Type column; review the extra columns against the approved contract or make them opt-in via Show Fields..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open Iteration Status list with Story and Defect rows.
+2. Verify there is no dedicated Type column.
+3. Verify US/DE formatted-ID prefix and type glyph identify each Work Item type.</x:v>
       </x:c>
       <x:c r="I40" s="38" t="str">
-        <x:v>List columns are checkbox, rank, ID, Type, Name, Schedule State, Iteration, Blocked, Plan Est, Task Est, To Do, Owner (P2-IS-FR-018).</x:v>
+        <x:v>Iteration Status has no dedicated Type column. Story/Defect type is conveyed by the US/DE ID prefix and type glyph in the identity cell.</x:v>
       </x:c>
       <x:c r="J40" s="38" t="str">
         <x:v>P2-IS-01</x:v>
@@ -3584,25 +3666,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L40" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M40" s="51" t="str">
-        <x:v>Populated Iteration Status list has no Type column.</x:v>
+        <x:v>Pass / Not a Defect. DevInt has no Type column and uses the approved identity prefix/glyph pattern.</x:v>
       </x:c>
       <x:c r="N40" s="51" t="str">
         <x:v>evidence/retest_2026-07-24/P2-IS-01-iteration-status.png</x:v>
       </x:c>
       <x:c r="O40" s="51" t="str">
-        <x:v>Add the approved Type column.</x:v>
+        <x:v>Closed by BA decision C3. Other extra columns are assessed separately.</x:v>
       </x:c>
       <x:c r="P40" s="51" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="Q40" s="51" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="R40" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Confirmed C3 — Closed / Not a Defect</x:v>
+      </x:c>
+      <x:c r="R40" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -3649,25 +3731,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L41" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M41" s="51" t="str">
-        <x:v>Iteration Status exposes a prohibited per-row Defects column.</x:v>
+        <x:v>Re-test 2026-08-09: Defects remains a summary metric and the per-row Defects column is absent.</x:v>
       </x:c>
       <x:c r="N41" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P2-IS-01-iteration-status.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/iteration-status</x:v>
       </x:c>
       <x:c r="O41" s="51" t="str">
-        <x:v>Remove the Defects column from current scope.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P41" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q41" s="51" t="str">
-        <x:v>Confirmed</x:v>
-      </x:c>
-      <x:c r="R41" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R41" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -3837,25 +3919,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L44" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M44" s="51" t="str">
-        <x:v>Team Status still exposes forbidden local Search tasks input.</x:v>
+        <x:v>Re-test 2026-08-09: Team Status no longer shows a local Search tasks input.</x:v>
       </x:c>
       <x:c r="N44" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P3-TS-01-team-status.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O44" s="51" t="str">
-        <x:v>Remove local search from Team Status.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P44" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q44" s="51" t="str">
-        <x:v>Gap Confirmed</x:v>
-      </x:c>
-      <x:c r="R44" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R44" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -3872,7 +3954,7 @@
         <x:v>P2</x:v>
       </x:c>
       <x:c r="E45" s="38" t="str">
-        <x:v>Filters/Show Fields/pagination controls</x:v>
+        <x:v>Team Status controls — C4 narrowed</x:v>
       </x:c>
       <x:c r="F45" s="38" t="str">
         <x:v>DevInt truy cập được và không có lỗi tải trang nghiêm trọng.
@@ -3882,18 +3964,13 @@
         <x:v>Project TEST; một Team có member và một Team không có member; Team Lead để trống khi case yêu cầu.</x:v>
       </x:c>
       <x:c r="H45" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở Track &gt; Team Status; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình Team Status, kiểm tra chức năng "Filters/Show Fields/pagination controls" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: DevInt shows a Filters button, a Show Fields button and full pagination (Rows per page, Page X of Y) copied from the Iteration Status/Backlog template..
-8. Kiểm tra hướng sửa đã chốt: Remove Filters/Show Fields/pagination from Team Status, or get explicit BA sign-off if this is an intentional deviation from the approved mockup..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open Team Status for an Iteration containing Tasks.
+2. Verify Filters and pagination are available.
+3. Verify local Search Tasks and Show Fields are absent.
+4. Apply a filter and change page; confirm Totals still reflect the full Iteration.</x:v>
       </x:c>
       <x:c r="I45" s="38" t="str">
-        <x:v>SRS section 7 screen mapping lists only the Iteration selector plus dense table with totals row; no Filters, Show Fields or pagination.</x:v>
+        <x:v>Filters and pagination are allowed. Local Search Tasks and Show Fields are absent. Totals always use all Tasks in the selected Iteration, independent of filters and page.</x:v>
       </x:c>
       <x:c r="J45" s="38" t="str">
         <x:v>P3-TS-01</x:v>
@@ -3902,25 +3979,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L45" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M45" s="51" t="str">
-        <x:v>Team Status still exposes forbidden Filters, Show Fields and rows-per-page pagination.</x:v>
+        <x:v>Re-test 2026-08-09: Filters and pagination remain, Show Fields is removed, and Totals show the full selected Iteration values (Capacity 60h, Estimate 4h, To Do 0h, Actuals 0h).</x:v>
       </x:c>
       <x:c r="N45" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P3-TS-01-team-status.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O45" s="51" t="str">
-        <x:v>Remove these inherited controls.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P45" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q45" s="51" t="str">
-        <x:v>Gap Confirmed</x:v>
-      </x:c>
-      <x:c r="R45" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R45" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -3967,25 +4044,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L46" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M46" s="51" t="str">
-        <x:v>Project &gt; Track &gt; Team Status breadcrumb is absent.</x:v>
+        <x:v>Re-test 2026-08-09: breadcrumb context shows Project &gt; Track &gt; Team Status.</x:v>
       </x:c>
       <x:c r="N46" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P3-TS-01-team-status.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O46" s="51" t="str">
-        <x:v>Implement approved breadcrumb hierarchy.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P46" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q46" s="51" t="str">
-        <x:v>Gap Confirmed</x:v>
-      </x:c>
-      <x:c r="R46" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R46" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -4099,22 +4176,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M48" s="51" t="str">
-        <x:v>Team Status task state is a three-segment control, not the required inline dropdown.</x:v>
+        <x:v>Re-test 2026-08-09: the screen shows member summary rows, but the existing Task row/control is not rendered, so the required inline State dropdown cannot be used.</x:v>
       </x:c>
       <x:c r="N48" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P3-TS-01-TA10.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O48" s="51" t="str">
-        <x:v>Replace with Defined / In-Progress / Completed dropdown.</x:v>
+        <x:v>DEV: render the Task row and its Defined / In-Progress / Completed dropdown.</x:v>
       </x:c>
       <x:c r="P48" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q48" s="51" t="str">
-        <x:v>Gap Confirmed</x:v>
-      </x:c>
-      <x:c r="R48" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R48" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -4164,22 +4241,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M49" s="51" t="str">
-        <x:v>Omitted Actuals displayed 0, but controlled test populated Estimate/To Do. A fully-empty Task is still needed to prove all defaults.</x:v>
+        <x:v>Re-test 2026-08-09: current Team Status totals and populated Task estimate values render, but there is no fully-empty Task row available to prove all three numeric defaults.</x:v>
       </x:c>
       <x:c r="N49" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P3-TS-01-TA10.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O49" s="51" t="str">
-        <x:v>Retest with a fully-empty Task.</x:v>
+        <x:v>Retest with a fully-empty Task after Task-row rendering is available.</x:v>
       </x:c>
       <x:c r="P49" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q49" s="51" t="str">
-        <x:v>Gap Confirmed</x:v>
-      </x:c>
-      <x:c r="R49" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R49" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -4229,22 +4306,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M50" s="51" t="str">
-        <x:v>Task controls render abbreviated/verb labels (D, I, Move to Completed), not exact catalog values.</x:v>
+        <x:v>Re-test 2026-08-09: no Task State control is rendered for the counted Task, so exact catalog labels cannot be verified or used.</x:v>
       </x:c>
       <x:c r="N50" s="51" t="str">
-        <x:v>evidence/retest_2026-07-24/P1-TASK-01-dashboard.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status</x:v>
       </x:c>
       <x:c r="O50" s="51" t="str">
-        <x:v>Use Defined / In-Progress / Completed labels.</x:v>
+        <x:v>DEV: render exact Defined / In-Progress / Completed Task State labels.</x:v>
       </x:c>
       <x:c r="P50" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q50" s="51" t="str">
-        <x:v>Gap Confirmed</x:v>
-      </x:c>
-      <x:c r="R50" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R50" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -4856,25 +4933,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L60" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M60" s="51" t="str">
-        <x:v>Workspace Settings shows read-only Slug and Workspace Admin identities, but no explicit single-company scope.</x:v>
+        <x:v>Re-test 2026-08-09: Workspace Settings now shows Slug, explicit Scope 'One company per workspace / Single company', and Workspace admin identities.</x:v>
       </x:c>
       <x:c r="N60" s="51" t="str">
-        <x:v>evidence/phase4_2026-07-24/P4-AUDIT-dev.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O60" s="51" t="str">
-        <x:v>Clarify scope in UI/SRS.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P60" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q60" s="51" t="str">
-        <x:v>BA Confirmed 2026-07-24</x:v>
-      </x:c>
-      <x:c r="R60" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R60" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -4902,18 +4979,13 @@
         <x:v>Dùng dữ liệu test riêng trong Project TEST. Nếu chưa có dữ liệu bắt buộc, ghi Blocked và nêu rõ dữ liệu còn thiếu.</x:v>
       </x:c>
       <x:c r="H61" s="38" t="str">
-        <x:v>1. Mở https://rally-dev.qnsc.vn/ và xác nhận đúng tài khoản/role của case.
-2. Chọn Workspace/Project/Team theo Test Data; ghi lại scope trước khi thao tác.
-3. Mở User Management; chụp trạng thái ban đầu nếu case liên quan UI, số liệu hoặc quyền.
-4. Thực hiện nghiệp vụ: Tại màn hình User Management, kiểm tra chức năng "List columns, role values and detail fields" theo Expected Result..
-5. Kiểm tra ngay UI, validation, quyền thao tác và các giá trị thay đổi so với Expected Result.
-6. Reload trang hoặc chuyển sang màn hình liên quan rồi quay lại; xác nhận dữ liệu và scope vẫn đúng.
-7. So sánh với lỗi/kết quả cũ: DevInt list replaces Phone number with Teams, contains Project Viewer/Workspace Member/blank roles, and non-admin detail has no Name/Phone or Remove User Access..
-8. Kiểm tra hướng sửa đã chốt: Align list/detail with SRS and mockup; remove unsupported roles; keep team allocation in detail without replacing the required Phone column; implement guarded Remove User Access..
-9. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
+        <x:v>1. Open User Management list.
+2. Verify columns are Name, Email, Role, Status and Last Login only.
+3. Open User Detail/Profile and verify Phone plus Team membership are available there.
+4. Verify approved roles and guarded Remove User Access.</x:v>
       </x:c>
       <x:c r="I61" s="38" t="str">
-        <x:v>List columns are Name, Email, Phone number, Role, Status and Last Login; roles are the approved three. Non-admin detail edits Name/Phone/Role/Status, keeps Email read-only and exposes Remove User Access.</x:v>
+        <x:v>User list contains Name, Email, Role, Status and Last Login; it excludes Phone and Teams. Phone is in Detail/Profile; Team membership is in User Detail/Team Members. Approved roles and guarded Remove User Access remain required.</x:v>
       </x:c>
       <x:c r="J61" s="38" t="str">
         <x:v>P4-SET-02</x:v>
@@ -4922,25 +4994,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L61" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M61" s="51" t="str">
-        <x:v>User Management has User, Email, Role, Status, Teams and Last Login. Phone is missing and Teams is unexpected.</x:v>
+        <x:v>Re-test 2026-08-09: user list now has User, Email, Role, Status and Last Login and no Teams/Phone columns. User Detail actions and approved role behavior are still not available from the list.</x:v>
       </x:c>
       <x:c r="N61" s="51" t="str">
-        <x:v>evidence/phase4_2026-07-24/P4-RBAC-dev.png; evidence/phase4_2026-07-24/P4-RBAC-mock.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O61" s="51" t="str">
-        <x:v>Align columns/fields to approved SRS.</x:v>
+        <x:v>DEV: complete User Detail, role and guarded access-removal behavior.</x:v>
       </x:c>
       <x:c r="P61" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q61" s="51" t="str">
-        <x:v>BA Confirmed 2026-07-24</x:v>
-      </x:c>
-      <x:c r="R61" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R61" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -4990,22 +5062,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M62" s="51" t="str">
-        <x:v>Audit Log displays technical auth.login.sso/access.role_elevated events and ID details, not business before/after detail.</x:v>
+        <x:v>Re-test 2026-08-09: Audit Log still mixes auth.login.sso/access.role_elevated technical events and entity IDs with business events.</x:v>
       </x:c>
       <x:c r="N62" s="51" t="str">
-        <x:v>evidence/phase4_2026-07-24/P4-AUDIT-dev.png; evidence/phase4_2026-07-24/P4-AUDIT-mock.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O62" s="51" t="str">
-        <x:v>Use business-readable event detail with before/after.</x:v>
+        <x:v>DEV: keep administrative mutations and business-readable before/after detail.</x:v>
       </x:c>
       <x:c r="P62" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q62" s="51" t="str">
-        <x:v>BA Confirmed 2026-07-24</x:v>
-      </x:c>
-      <x:c r="R62" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R62" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -5052,25 +5124,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L63" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M63" s="51" t="str">
-        <x:v>Selecting Deactive on Pegasus saved immediately with Status updated; no target-specific confirmation. BA-approved restore returned Pegasus to Active.</x:v>
+        <x:v>Re-test 2026-08-09: changing Pegasus to Deactive now opens a target-specific 'Archive team' confirmation. Typed confirmation for Remove User Access was not available to verify.</x:v>
       </x:c>
       <x:c r="N63" s="51" t="str">
-        <x:v>evidence/phase4_2026-07-24/P4-AUDIT-dev.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O63" s="51" t="str">
-        <x:v>Require confirmation before destructive Team status action.</x:v>
+        <x:v>Team branch fixed; retest guarded User-access removal when User Detail is implemented.</x:v>
       </x:c>
       <x:c r="P63" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q63" s="51" t="str">
-        <x:v>BA Confirmed 2026-07-24</x:v>
-      </x:c>
-      <x:c r="R63" s="56" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R63" s="56" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -5117,25 +5189,25 @@
         <x:v>Still Open</x:v>
       </x:c>
       <x:c r="L64" s="53" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M64" s="53" t="str">
-        <x:v>Notification Preferences remains in Settings navigation despite approved Phase 4 scope removing it.</x:v>
+        <x:v>Re-test 2026-08-09: Notification Preferences is absent from Settings navigation.</x:v>
       </x:c>
       <x:c r="N64" s="53" t="str">
-        <x:v>evidence/phase4_2026-07-24/P4-AUDIT-dev.png</x:v>
+        <x:v>https://rally-dev.qnsc.vn/settings</x:v>
       </x:c>
       <x:c r="O64" s="53" t="str">
-        <x:v>Remove from current scope navigation.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P64" s="53" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q64" s="53" t="str">
-        <x:v>BA Confirmed 2026-07-24</x:v>
-      </x:c>
-      <x:c r="R64" s="57" t="str">
-        <x:v>2026-08-05</x:v>
+        <x:v>Pending BA confirmation</x:v>
+      </x:c>
+      <x:c r="R64" s="57" t="n">
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -5181,22 +5253,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M65" t="str">
-        <x:v>Hieu appeared in Team Status before belonging to Pegasus. After Hieu was added, Settings &gt; Teams and Team Status both showed Anh and Hieu, but the US-1 Owner dropdown still showed only No Entry and Anh.</x:v>
+        <x:v>Re-test 2026-08-09: Settings &gt; Teams lists only Anh in Pegasus, while Team Status still groups Hieu with 1 Task. Work Item Owner choices also omit Hieu.</x:v>
       </x:c>
       <x:c r="N65" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/team-status; https://rally-dev.qnsc.vn/settings; https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O65" t="str">
-        <x:v>Use one current Team-membership source for Team Status and Owner selectors, and refresh/invalidate membership caches after add/remove. Existing Task-owner treatment when a member is removed remains Pending BA.</x:v>
+        <x:v>DEV: use one current Team-membership source and invalidate stale Team Status membership.</x:v>
       </x:c>
       <x:c r="P65" t="str">
-        <x:v>BA + Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q65" t="str">
-        <x:v>Bug confirmed; removal behavior pending</x:v>
+        <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R65" s="92" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5264,7 +5336,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>78 approved mockup/UAT scenarios. Previous mockup Pass does not replace deployed-product verification.</x:v>
+        <x:v>Historical Phase 5 deployed-product results. Current Project authorization must be re-tested against Current Access Baseline; former role wording is retained only as execution history.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -5508,22 +5580,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M7" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: inline-edit controls remain present on Feature rows, but a complete Project-change validity cycle was not executable with the single Project dataset.</x:v>
       </x:c>
       <x:c r="N7" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O7" s="51" t="str">
-        <x:v>Workspace Admin controls were inspected, but not every inline field mutation was executed.</x:v>
+        <x:v>Retest Feature Project change with a second Project; Epic restrictions remain data-dependent.</x:v>
       </x:c>
       <x:c r="P7" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q7" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R7" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5766,22 +5838,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M11" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: only Project TEST and its release data are available, so cross-Project Release filtering cannot be exercised.</x:v>
       </x:c>
       <x:c r="N11" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O11" s="51" t="str">
-        <x:v>Only Project TEST was available; cross-Project Release filtering was not exercised.</x:v>
+        <x:v>Needs a second Project with a distinct Release.</x:v>
       </x:c>
       <x:c r="P11" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q11" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R11" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -5827,25 +5899,25 @@
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="L12" s="51" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M12" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Create with details created exactly FE-4 and navigated directly to its Feature Detail page.</x:v>
       </x:c>
       <x:c r="N12" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio/019fe657-7173-7e33-b737-2edf1f4b6395</x:v>
       </x:c>
       <x:c r="O12" s="51" t="str">
-        <x:v>Create was tested; Create with details was not executed.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P12" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q12" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R12" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -5894,22 +5966,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M13" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: FE-4 Description saved and persisted after reload. Attachment persistence was not exercised.</x:v>
       </x:c>
       <x:c r="N13" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio/019fe657-7173-7e33-b737-2edf1f4b6395</x:v>
       </x:c>
       <x:c r="O13" s="51" t="str">
-        <x:v>Backing fields were visible; full rich-text and attachment persistence was not exercised.</x:v>
+        <x:v>Text persistence passes; attachment branch still needs a controlled file.</x:v>
       </x:c>
       <x:c r="P13" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q13" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R13" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -6022,22 +6094,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M15" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: current data does not expose a newly archived Feature/Epic branch for a fresh Add Item absence check.</x:v>
       </x:c>
       <x:c r="N15" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O15" s="51" t="str">
-        <x:v>Archived read-only state was observed; Children-tab Add Item absence was not reopened separately.</x:v>
+        <x:v>Retest on an archived portfolio item with preserved children/history.</x:v>
       </x:c>
       <x:c r="P15" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q15" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R15" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -6208,22 +6280,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M18" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Children counts and tabs are present, but Task expansion and the complete Backlog-style grid control set could not be exercised with the current child dataset.</x:v>
       </x:c>
       <x:c r="N18" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio/019fd5d9-9137-731a-aa13-aee2e012ac5d</x:v>
       </x:c>
       <x:c r="O18" s="51" t="str">
-        <x:v>Children grid and routing were checked; Task expansion and all grid controls were not exhaustively exercised.</x:v>
+        <x:v>Needs a Feature containing Story/Defect and Task rows.</x:v>
       </x:c>
       <x:c r="P18" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q18" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R18" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -6397,22 +6469,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M21" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: the previously linked child remains visible by count, but a fresh child-create rollup cycle could not be completed from the current Children tab interaction.</x:v>
       </x:c>
       <x:c r="N21" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio/019fd5d9-9137-731a-aa13-aee2e012ac5d</x:v>
       </x:c>
       <x:c r="O21" s="51" t="str">
-        <x:v>US-3 persisted and linked to FE-1, but child count/rollup stayed stale until reload.</x:v>
+        <x:v>Retest immediate child count/rollup refresh after creating a Feature-linked Work Item.</x:v>
       </x:c>
       <x:c r="P21" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q21" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R21" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -6460,22 +6532,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M22" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: only one Project is available, so invalid Feature clearing after Project change remains unverified.</x:v>
       </x:c>
       <x:c r="N22" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O22" s="51" t="str">
-        <x:v>Feature assignment persisted; invalid Feature clearing after Project change was not tested.</x:v>
+        <x:v>Needs two Projects with distinct active Features.</x:v>
       </x:c>
       <x:c r="P22" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q22" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R22" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -7078,22 +7150,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M32" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Feature rollups render on the available simple dataset, but multi-level Epic denominator branches remain unavailable.</x:v>
       </x:c>
       <x:c r="N32" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O32" s="51" t="str">
-        <x:v>Epic child presence was confirmed; formula coverage used only the available zero/simple denominator data.</x:v>
+        <x:v>Needs controlled Epic &gt; multiple Features &gt; leaf Story/Defect estimates.</x:v>
       </x:c>
       <x:c r="P32" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q32" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R32" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -7327,22 +7399,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M36" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: bulk selection/actions remain visible; destructive archive and active-child blocking were not executed on shared data.</x:v>
       </x:c>
       <x:c r="N36" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O36" s="51" t="str">
-        <x:v>Root checkbox/bulk controls were visible; destructive bulk action was not executed.</x:v>
+        <x:v>Retest with disposable Epic/Feature records.</x:v>
       </x:c>
       <x:c r="P36" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q36" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R36" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -7390,22 +7462,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M37" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: current dataset still lacks multiple Feature children under one Epic for a rank comparison.</x:v>
       </x:c>
       <x:c r="N37" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/portfolio</x:v>
       </x:c>
       <x:c r="O37" s="51" t="str">
-        <x:v>A single child Feature was available, so multi-child rank display was not compared.</x:v>
+        <x:v>Needs one Epic with at least two Feature children.</x:v>
       </x:c>
       <x:c r="P37" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q37" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R37" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -7825,22 +7897,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M44" s="51" t="str">
-        <x:v>Fail. Draft Team Capacity is text only ('Not entered' or '30 points'); there is no manual inline editor. Capacity can only be populated through Forecast.</x:v>
+        <x:v>Re-test 2026-08-09: Team Capacity still renders '30 points' as text; only Forecast capacity is actionable and no Draft inline editor is present.</x:v>
       </x:c>
       <x:c r="N44" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O44" s="51" t="str">
-        <x:v>Restore Draft-only manual Capacity editing without changing allocation or Feature estimates.</x:v>
+        <x:v>DEV: restore Draft-only manual Capacity editing.</x:v>
       </x:c>
       <x:c r="P44" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q44" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R44" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -7889,22 +7961,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M45" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Pegasus is present as the single Plan Team. Remove-and-restore cannot be safely validated without a second disposable Team/allocation.</x:v>
       </x:c>
       <x:c r="N45" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O45" s="51" t="str">
-        <x:v>Add Team was tested. Remove-and-restore was not repeated because Pegasus owns the active allocation.</x:v>
+        <x:v>Needs a second disposable Team.</x:v>
       </x:c>
       <x:c r="P45" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q45" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R45" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -8014,22 +8086,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M47" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: only one usable Team exists, so split allocation and its default-zero row cannot be exercised.</x:v>
       </x:c>
       <x:c r="N47" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O47" s="51" t="str">
-        <x:v>Single-Team allocation was tested; split allocation requires a second usable Team.</x:v>
+        <x:v>Needs a second usable Team.</x:v>
       </x:c>
       <x:c r="P47" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q47" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R47" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -8201,22 +8273,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M50" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Teams and Features views are present; independent sort persistence could not be completed because the Teams-tab interaction timed out in the current session.</x:v>
       </x:c>
       <x:c r="N50" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O50" s="51" t="str">
-        <x:v>Both tabs worked; independent sort persistence was not fully exercised.</x:v>
+        <x:v>Retest both tab sort states after UI interaction stabilizes.</x:v>
       </x:c>
       <x:c r="P50" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q50" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R50" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -8264,22 +8336,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M51" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: allocation estimate and Rank view remain visible, but split-Team and capacity-cutline branches lack the required data.</x:v>
       </x:c>
       <x:c r="N51" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O51" s="51" t="str">
-        <x:v>Allocation and estimate display were tested; split allocation and capacity cutline branches were not.</x:v>
+        <x:v>Needs multiple ranked Features and split allocation.</x:v>
       </x:c>
       <x:c r="P51" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q51" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R51" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -8450,22 +8522,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M54" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: the current shared plan remains Draft; publish mismatch and child non-cascade branches were not repeated.</x:v>
       </x:c>
       <x:c r="N54" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O54" s="51" t="str">
-        <x:v>Visibility-only Publish, Unpublish and matching-date full Publish passed; child non-cascade/mismatch branches remain.</x:v>
+        <x:v>Retest with a disposable Draft plan and child Work Items.</x:v>
       </x:c>
       <x:c r="P54" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q54" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R54" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -9019,22 +9091,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M63" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Estimated shows Allocated 8 as the selected tier; Refined and Preliminary fallback branches are not both available.</x:v>
       </x:c>
       <x:c r="N63" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O63" s="51" t="str">
-        <x:v>Manual allocation precedence was observed; Refined and Preliminary fallback branches were not both exercised.</x:v>
+        <x:v>Needs controlled Features for each fallback tier.</x:v>
       </x:c>
       <x:c r="P63" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q63" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R63" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -9145,22 +9217,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M65" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Dependencies remains a dash placeholder; cross-Team origin attribution cannot be tested with one Team.</x:v>
       </x:c>
       <x:c r="N65" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O65" s="51" t="str">
-        <x:v>Dependencies placeholder was present; cross-Team origin attribution requires a second Team.</x:v>
+        <x:v>Needs split allocation across a second Team.</x:v>
       </x:c>
       <x:c r="P65" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q65" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R65" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -9273,22 +9345,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M67" s="51" t="str">
-        <x:v>Partial. Remove from Plan persisted and FE-3 disappeared after reload, but the row and count stayed stale immediately after the success toast.</x:v>
+        <x:v>Re-test 2026-08-09: no disposable allocated Feature was removed from the shared plan; the prior immediate-refresh gap therefore remains open for regression.</x:v>
       </x:c>
       <x:c r="N67" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O67" s="51" t="str">
-        <x:v>DEV should refetch/invalidate the plan immediately after Remove from Plan.</x:v>
+        <x:v>Retest Remove from Plan with a disposable Feature and verify immediate counters.</x:v>
       </x:c>
       <x:c r="P67" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q67" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R67" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -9401,22 +9473,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M69" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Complete, Rollup, Estimated and Capacity totals render; no child status transition was executed to prove Complete decreases.</x:v>
       </x:c>
       <x:c r="N69" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O69" s="51" t="str">
-        <x:v>Basic totals were visible; a child status transition was not executed in this Phase 5 run.</x:v>
+        <x:v>Needs a Feature with controlled child Plan Estimates/statuses.</x:v>
       </x:c>
       <x:c r="P69" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q69" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R69" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -9515,7 +9587,7 @@
 7. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
       </x:c>
       <x:c r="I71" s="38" t="str">
-        <x:v>Grid columns are Rank, ID, Name, Planned Team Assignment, Team, Dependencies, Complete, Rollup, Estimated; ID shows only the Feature ID with no type badge; there is no grid-level progress bar, no State/Planned Team header, and metrics align to the right. Split Feature allocation subrows show Team slices. The row settings menu overlays the grid and contains only Allocate and Remove from Plan.</x:v>
+        <x:v>Grid columns are Rank, ID, Name, Planned Team Assignment, Team, Dependencies, Rollup, Estimated, Complete. ID uses the Feature prefix without a separate Type column; metrics align right and split rows show Team slices.</x:v>
       </x:c>
       <x:c r="J71" s="38" t="str">
         <x:v>Phase 5/02_Capacity_Planning/SRS.md</x:v>
@@ -9524,25 +9596,25 @@
         <x:v>Pass 2026-07-28. Browser smoke on CP-001 confirmed the new headers, FE-318 parent total 0 / 6 / 8, allocation subrows Data &amp; Reporting 0 / 6 / 5 and Core Platform 0 / 0 / 3, no Feature-grid progress-bar node beyond the plan header bar, ID rendered as FE-318 without the type badge, and settings menu items Allocate / Remove from Plan only. Build passed with only the standard Vite chunk-size warning.</x:v>
       </x:c>
       <x:c r="L71" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M71" s="51" t="str">
-        <x:v>Fail. Features grid order is Dependencies, Rollup, Estimated, Complete instead of Dependencies, Complete, Rollup, Estimated.</x:v>
+        <x:v>Pass / Not a Defect. DevInt order Dependencies, Rollup, Estimated, Complete is the C8-confirmed baseline.</x:v>
       </x:c>
       <x:c r="N71" s="51" t="str">
         <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
       </x:c>
       <x:c r="O71" s="51" t="str">
-        <x:v>Reorder the Features grid metrics to Complete, Rollup, Estimated.</x:v>
+        <x:v>Closed by BA decision C8. SRS/mockup corrected; no DEV reorder required.</x:v>
       </x:c>
       <x:c r="P71" s="51" t="str">
         <x:v>Codex — Workspace Admin</x:v>
       </x:c>
       <x:c r="Q71" s="51" t="str">
-        <x:v>Pending BA confirmation</x:v>
+        <x:v>Confirmed C8 — Closed / Not a Defect</x:v>
       </x:c>
       <x:c r="R71" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -9591,22 +9663,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M72" s="51" t="str">
-        <x:v>Fail. Selecting Pegasus in Planned Team Assignment changes counters but the selector remains Not assigned, including after reload.</x:v>
+        <x:v>Re-test 2026-08-09: FE-2 is listed under Pegasus allocation but Planned Team Assignment still displays Not assigned after reload.</x:v>
       </x:c>
       <x:c r="N72" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O72" s="51" t="str">
-        <x:v>Persist and render quick Planned Team from the shared allocation ledger.</x:v>
+        <x:v>DEV: persist/render Planned Team from the shared allocation ledger.</x:v>
       </x:c>
       <x:c r="P72" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q72" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R72" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -9655,22 +9727,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M73" s="51" t="str">
-        <x:v>Partial. The main available branch worked, but one or more branches could not be completed with the current scope/data.</x:v>
+        <x:v>Re-test 2026-08-09: Rank, actions, Breakdown and Team Capacity rail remain present; warning branches still lack suitable exceed/missing-estimate data.</x:v>
       </x:c>
       <x:c r="N73" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O73" s="51" t="str">
-        <x:v>Rank, actions and Breakdown passed; exceed-warning branch lacked suitable data.</x:v>
+        <x:v>Needs controlled warning-trigger data.</x:v>
       </x:c>
       <x:c r="P73" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q73" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R73" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -9719,22 +9791,22 @@
         <x:v>Fail</x:v>
       </x:c>
       <x:c r="M74" s="51" t="str">
-        <x:v>Fail. Planned Team never renders as assigned, so the one-Team selector does not expose a usable Unassign flow.</x:v>
+        <x:v>Re-test 2026-08-09: Features tab toolbar is aligned, but Planned Team remains Not assigned, so Unassign cannot be offered or verified.</x:v>
       </x:c>
       <x:c r="N74" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O74" s="51" t="str">
-        <x:v>Fix P5-CP-032 first, then verify Unassign clears the Team while retaining the Feature in the plan.</x:v>
+        <x:v>Fix P5-CP-032 first, then verify Unassign retains the Feature in plan.</x:v>
       </x:c>
       <x:c r="P74" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q74" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R74" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -9783,22 +9855,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M75" s="51" t="str">
-        <x:v>Partial. Matching-date full Publish passed and wrote RE-1 plus both dates to FE-2; mismatching Plan-vs-Release dates were not tested.</x:v>
+        <x:v>Re-test 2026-08-09: current plan/release data does not provide a disposable mismatching-date publish branch.</x:v>
       </x:c>
       <x:c r="N75" s="51" t="str">
-        <x:v>DevInt browser retest 2026-08-06; controlled P56-AUDIT data. Detail: 07_Testing Plan/Codex_audit_06_tracker.md &gt; Phase 5 DevInt Execution Results.</x:v>
+        <x:v>https://rally-dev.qnsc.vn/capacity-planning/41d10dd3-6392-47c0-8972-bc4e521d319e</x:v>
       </x:c>
       <x:c r="O75" s="51" t="str">
-        <x:v>Retest the mismatching Plan-date versus Release-date advisory branch.</x:v>
+        <x:v>Needs a disposable Plan whose dates mismatch its Release.</x:v>
       </x:c>
       <x:c r="P75" s="51" t="str">
-        <x:v>Codex — Workspace Admin</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q75" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R75" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -10667,22 +10739,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M9" s="51" t="str">
-        <x:v>Explicit empty states were confirmed in Reports and Release Tracking; a second empty Project is unavailable.</x:v>
+        <x:v>Re-test 2026-08-09: explicit empty states still render; a second empty Project is unavailable to prove no cross-Project reuse.</x:v>
       </x:c>
       <x:c r="N9" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports; https://rally-dev.qnsc.vn/release-tracking</x:v>
       </x:c>
       <x:c r="O9" s="51" t="str">
-        <x:v>Follow-up: Explicit empty states were confirmed in Reports and Release Tracking; a second empty Project is unavailable.</x:v>
+        <x:v>Needs a second Project with no Phase 6 data.</x:v>
       </x:c>
       <x:c r="P9" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q9" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R9" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10727,25 +10799,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L10" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M10" s="51" t="str">
-        <x:v>Reports and Release Tracking reset the selected view/filter after reload.</x:v>
+        <x:v>Re-test 2026-08-09: Reports Type=Velocity and Window=Last 5 persisted after reload; Release Tracking Chart Unit=Count and Unparented bucket also persisted.</x:v>
       </x:c>
       <x:c r="N10" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports; https://rally-dev.qnsc.vn/release-tracking</x:v>
       </x:c>
       <x:c r="O10" s="51" t="str">
-        <x:v>DEV: preserve selected Reports Type/window and Release Tracking Chart Unit/bucket across reload.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P10" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q10" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R10" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10915,22 +10987,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M13" s="51" t="str">
-        <x:v>Rank, ID and Team sort states changed correctly; column resizing was not executed.</x:v>
+        <x:v>Re-test 2026-08-09: Rank/ID/Name/Team sorting controls and readable names remain present; column resize was not executed.</x:v>
       </x:c>
       <x:c r="N13" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/release-tracking</x:v>
       </x:c>
       <x:c r="O13" s="51" t="str">
-        <x:v>Follow-up: Rank, ID and Team sort states changed correctly; column resizing was not executed.</x:v>
+        <x:v>Retest drag resize on a stable browser session.</x:v>
       </x:c>
       <x:c r="P13" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q13" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R13" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -11162,22 +11234,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M17" s="51" t="str">
-        <x:v>Completed is excluded and Accepted is included; Release-state branch lacks controlled data.</x:v>
+        <x:v>Re-test 2026-08-09: Completed US-4 contributes 0 accepted, confirming Completed is excluded. A Release-state Work Item is still unavailable.</x:v>
       </x:c>
       <x:c r="N17" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/release-tracking</x:v>
       </x:c>
       <x:c r="O17" s="51" t="str">
-        <x:v>Follow-up: Completed is excluded and Accepted is included; Release-state branch lacks controlled data.</x:v>
+        <x:v>Needs a Release-state Work Item in the selected Project/Team.</x:v>
       </x:c>
       <x:c r="P17" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q17" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R17" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -11596,22 +11668,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M24" s="51" t="str">
-        <x:v>Valid Release empty-bucket messaging passed; no second Project without Releases is available.</x:v>
+        <x:v>Re-test 2026-08-09: empty snapshot gaps are displayed as 'no data'; no second Project without Releases is available for the no-Release state.</x:v>
       </x:c>
       <x:c r="N24" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/release-tracking</x:v>
       </x:c>
       <x:c r="O24" s="51" t="str">
-        <x:v>Follow-up: Valid Release empty-bucket messaging passed; no second Project without Releases is available.</x:v>
+        <x:v>Needs a Project with no Releases.</x:v>
       </x:c>
       <x:c r="P24" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q24" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R24" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -12469,7 +12541,7 @@
 7. Ghi Actual Result, chọn Current Status, điền Evidence và Gap/Comment trong chính dòng case.</x:v>
       </x:c>
       <x:c r="I38" s="38" t="str">
-        <x:v>Bars, trend and Last/Best/Worst averages use selected window; default is Last 5</x:v>
+        <x:v>Bars, trend and Last/Best/Worst averages use the selected window; default is Last 10. User can toggle Last 5/Last 10 and the selection persists after reload.</x:v>
       </x:c>
       <x:c r="J38" s="38" t="str">
         <x:v>Phase 6/03_Velocity_Chart/SRS.md</x:v>
@@ -12478,25 +12550,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L38" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M38" s="51" t="str">
-        <x:v>Control works, but default is Last 10 instead of the required Last 5.</x:v>
+        <x:v>Pass / Not a Defect. DevInt default Last 10 matches C7; the 5/10 selection must persist.</x:v>
       </x:c>
       <x:c r="N38" s="51" t="str">
         <x:v>../Codex_audit_06_tracker.md</x:v>
       </x:c>
       <x:c r="O38" s="51" t="str">
-        <x:v>DEV: default Velocity to Last 5 sprints and preserve the selected window.</x:v>
+        <x:v>Closed by BA decision C7. Preserve the existing default and regression-test selection persistence.</x:v>
       </x:c>
       <x:c r="P38" s="51" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="Q38" s="51" t="str">
-        <x:v>Pending BA confirmation</x:v>
+        <x:v>Confirmed C7 — Closed / Not a Defect</x:v>
       </x:c>
       <x:c r="R38" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -13474,25 +13546,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L54" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="M54" s="51" t="str">
-        <x:v>Create with details silently created duplicate/orphan Work Items while leaving the dialog open and showing no confirmation.</x:v>
+        <x:v>Re-test 2026-08-09: one Create with details submission created exactly US-7, closed the dialog, navigated to detail, and Backlog search returned 1–1 of 1.</x:v>
       </x:c>
       <x:c r="N54" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/US-7; https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O54" s="51" t="str">
-        <x:v>DEV: one submission must create exactly one Work Item; close/navigate after success and disable duplicate submission while saving.</x:v>
+        <x:v>Resolved in current DevInt.</x:v>
       </x:c>
       <x:c r="P54" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q54" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R54" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -13538,25 +13610,25 @@
         <x:v>New production acceptance scenario</x:v>
       </x:c>
       <x:c r="L55" s="51" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="M55" s="51" t="str">
-        <x:v>Work Item state update did not persist/mirror reliably; Schedule/Flow returned to Idea after reload and reporting did not count it as accepted.</x:v>
+        <x:v>Re-test 2026-08-09: US-7 Flow State=Accepted saved, mirrored to Schedule State, persisted after reload, and appeared consistently in Backlog. Parent/Iteration/Release rollups were not attached to this disposable item.</x:v>
       </x:c>
       <x:c r="N55" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/item/US-7; https://rally-dev.qnsc.vn/backlog</x:v>
       </x:c>
       <x:c r="O55" s="51" t="str">
-        <x:v>DEV: persist Work Item states and enforce two-way Schedule State/Flow State mirroring before report totals refresh.</x:v>
+        <x:v>Core state persistence/mirroring fixed; retest full parent/Iteration/Release rollup chain.</x:v>
       </x:c>
       <x:c r="P55" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q55" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R55" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -13604,22 +13676,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M56" s="51" t="str">
-        <x:v>Project/Team scope changed correctly; only one Release and one Iteration prevent cross-context validation.</x:v>
+        <x:v>Re-test 2026-08-09: Project/Team scoping remains consistent, but only one Release and one Iteration are available for cross-context invalidation.</x:v>
       </x:c>
       <x:c r="N56" s="51" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/backlog; https://rally-dev.qnsc.vn/release-tracking</x:v>
       </x:c>
       <x:c r="O56" s="51" t="str">
-        <x:v>Follow-up: Project/Team scope changed correctly; only one Release and one Iteration prevent cross-context validation.</x:v>
+        <x:v>Needs multiple Releases/Iterations/Projects.</x:v>
       </x:c>
       <x:c r="P56" s="51" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q56" s="51" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R56" s="56" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -13667,22 +13739,22 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="M57" s="53" t="str">
-        <x:v>Record data persisted in several flows, but report filters reset on reload; sign-out/in was not repeated.</x:v>
+        <x:v>Re-test 2026-08-09: record values and Phase 6 view selections persisted after reload. A sign-out/sign-in authorization cycle was not repeated.</x:v>
       </x:c>
       <x:c r="N57" s="53" t="str">
-        <x:v>../Codex_audit_06_tracker.md</x:v>
+        <x:v>https://rally-dev.qnsc.vn/reports; https://rally-dev.qnsc.vn/release-tracking; https://rally-dev.qnsc.vn/item/US-7</x:v>
       </x:c>
       <x:c r="O57" s="53" t="str">
-        <x:v>Follow-up: Record data persisted in several flows, but report filters reset on reload; sign-out/in was not repeated.</x:v>
+        <x:v>Persistence branch passes; authentication-cycle branch remains.</x:v>
       </x:c>
       <x:c r="P57" s="53" t="str">
-        <x:v>Codex</x:v>
+        <x:v>Codex DevInt re-test</x:v>
       </x:c>
       <x:c r="Q57" s="53" t="str">
         <x:v>Pending BA confirmation</x:v>
       </x:c>
       <x:c r="R57" s="57" t="n">
-        <x:v>46240</x:v>
+        <x:v>46243</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14900,16 +14972,16 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="F46" s="83" t="str">
-        <x:v>Fail</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="G46" s="83" t="str">
         <x:v>../Codex_audit_06_tracker.md</x:v>
       </x:c>
       <x:c r="H46" s="83" t="str">
-        <x:v>P6-GAP-003</x:v>
+        <x:v>N/A — C7 reconciliation</x:v>
       </x:c>
       <x:c r="I46" s="73" t="str">
-        <x:v>Control works, but default is Last 10 instead of the required Last 5.</x:v>
+        <x:v>BA confirmed default Last 10 with a Last 5/Last 10 toggle and persisted selection. Previous failure reclassified as Not a Defect.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -15459,15 +15531,33 @@
       </x:c>
     </x:row>
     <x:row r="67">
-      <x:c r="A67" s="86"/>
-      <x:c r="B67" s="83"/>
-      <x:c r="C67" s="83"/>
-      <x:c r="D67" s="83"/>
-      <x:c r="E67" s="83"/>
-      <x:c r="F67" s="83"/>
-      <x:c r="G67" s="83"/>
-      <x:c r="H67" s="83"/>
-      <x:c r="I67" s="73"/>
+      <x:c r="A67" s="86" t="n">
+        <x:v>46243</x:v>
+      </x:c>
+      <x:c r="B67" s="83" t="str">
+        <x:v>FAIL-PARTIAL-RETEST-20260809</x:v>
+      </x:c>
+      <x:c r="C67" s="83" t="str">
+        <x:v>https://rally-dev.qnsc.vn/</x:v>
+      </x:c>
+      <x:c r="D67" s="83" t="str">
+        <x:v>QNSC / TEST / Pegasus</x:v>
+      </x:c>
+      <x:c r="E67" s="83" t="str">
+        <x:v>Codex DevInt re-test</x:v>
+      </x:c>
+      <x:c r="F67" s="83" t="str">
+        <x:v>11 Pass / 31 Partial / 9 Fail</x:v>
+      </x:c>
+      <x:c r="G67" s="83" t="str">
+        <x:v>Codex_audit_06_tracker.md</x:v>
+      </x:c>
+      <x:c r="H67" s="83" t="str">
+        <x:v>9 Fail</x:v>
+      </x:c>
+      <x:c r="I67" s="73" t="str">
+        <x:v>Re-tested 51 prior Fail/Partial scenarios; existing Blocked scenarios were excluded.</x:v>
+      </x:c>
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="86"/>
@@ -16944,4 +17034,507 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="20" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="25" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="45" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="30" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="36" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" hidden="0" customHeight="1">
+      <x:c r="A1" s="95" t="str">
+        <x:v>Mini Rally Current Project Access Baseline</x:v>
+      </x:c>
+      <x:c r="B1" s="95"/>
+      <x:c r="C1" s="95"/>
+      <x:c r="D1" s="95"/>
+      <x:c r="E1" s="95"/>
+      <x:c r="F1" s="95"/>
+      <x:c r="G1" s="95"/>
+      <x:c r="H1" s="95"/>
+    </x:row>
+    <x:row r="2" ht="36" hidden="0" customHeight="1">
+      <x:c r="A2" s="99" t="str">
+        <x:v>Approved 2026-08-10. This sheet supersedes former global Project Admin/Project Member/Project Viewer role assumptions. Historical execution results remain unchanged.</x:v>
+      </x:c>
+      <x:c r="B2" s="99"/>
+      <x:c r="C2" s="99"/>
+      <x:c r="D2" s="99"/>
+      <x:c r="E2" s="99"/>
+      <x:c r="F2" s="99"/>
+      <x:c r="G2" s="99"/>
+      <x:c r="H2" s="99"/>
+    </x:row>
+    <x:row r="3" ht="34" hidden="0" customHeight="1">
+      <x:c r="A3" s="99" t="str">
+        <x:v>Company role: Workspace Admin only. All other authorization is assigned independently per Project as Admin, Editor, Viewer, or No Access.</x:v>
+      </x:c>
+      <x:c r="B3" s="99"/>
+      <x:c r="C3" s="99"/>
+      <x:c r="D3" s="99"/>
+      <x:c r="E3" s="99"/>
+      <x:c r="F3" s="99"/>
+      <x:c r="G3" s="99"/>
+      <x:c r="H3" s="99"/>
+    </x:row>
+    <x:row r="4" ht="30" hidden="0" customHeight="1">
+      <x:c r="A4" s="104" t="str">
+        <x:v>Role / Access Level</x:v>
+      </x:c>
+      <x:c r="B4" s="104" t="str">
+        <x:v>Assignment Scope</x:v>
+      </x:c>
+      <x:c r="C4" s="104" t="str">
+        <x:v>Team Scope</x:v>
+      </x:c>
+      <x:c r="D4" s="104" t="str">
+        <x:v>Delivery Capabilities</x:v>
+      </x:c>
+      <x:c r="E4" s="104" t="str">
+        <x:v>Structural Settings</x:v>
+      </x:c>
+      <x:c r="F4" s="104" t="str">
+        <x:v>Project Visibility</x:v>
+      </x:c>
+      <x:c r="G4" s="104" t="str">
+        <x:v>Effective Time</x:v>
+      </x:c>
+      <x:c r="H4" s="104" t="str">
+        <x:v>Test State</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A5" s="115" t="str">
+        <x:v>Workspace Admin</x:v>
+      </x:c>
+      <x:c r="B5" s="112" t="str">
+        <x:v>Company-wide; assigned internally</x:v>
+      </x:c>
+      <x:c r="C5" s="112" t="str">
+        <x:v>Not a Project or Team member</x:v>
+      </x:c>
+      <x:c r="D5" s="112" t="str">
+        <x:v>Full access across all Projects</x:v>
+      </x:c>
+      <x:c r="E5" s="112" t="str">
+        <x:v>CRUD Projects/Teams; manage users and Project access</x:v>
+      </x:c>
+      <x:c r="F5" s="112" t="str">
+        <x:v>All Projects</x:v>
+      </x:c>
+      <x:c r="G5" s="112" t="str">
+        <x:v>Access changes: next sign-in; company disable/removal: next refresh</x:v>
+      </x:c>
+      <x:c r="H5" s="118" t="str">
+        <x:v>Approved baseline</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="158.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A6" s="116" t="str">
+        <x:v>Admin</x:v>
+      </x:c>
+      <x:c r="B6" s="113" t="str">
+        <x:v>Per assigned Project</x:v>
+      </x:c>
+      <x:c r="C6" s="113" t="str">
+        <x:v>All Teams in that Project</x:v>
+      </x:c>
+      <x:c r="D6" s="113" t="str">
+        <x:v>Full delivery administration, including planning, tracking, quality, portfolio, capacity, and reports</x:v>
+      </x:c>
+      <x:c r="E6" s="113" t="str">
+        <x:v>Read-only Project details, Teams, Users &amp; Permissions</x:v>
+      </x:c>
+      <x:c r="F6" s="113" t="str">
+        <x:v>Assigned Project only</x:v>
+      </x:c>
+      <x:c r="G6" s="113" t="str">
+        <x:v>Next sign-in</x:v>
+      </x:c>
+      <x:c r="H6" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="132" hidden="0" customHeight="1">
+      <x:c r="A7" s="116" t="str">
+        <x:v>Editor</x:v>
+      </x:c>
+      <x:c r="B7" s="113" t="str">
+        <x:v>Per assigned Project</x:v>
+      </x:c>
+      <x:c r="C7" s="113" t="str">
+        <x:v>Explicit Teams only</x:v>
+      </x:c>
+      <x:c r="D7" s="113" t="str">
+        <x:v>CRUD US/DE/Task and Quality Defects in assigned Teams; update Iteration Status</x:v>
+      </x:c>
+      <x:c r="E7" s="113" t="str">
+        <x:v>No structural administration</x:v>
+      </x:c>
+      <x:c r="F7" s="113" t="str">
+        <x:v>Assigned Project and Teams only</x:v>
+      </x:c>
+      <x:c r="G7" s="113" t="str">
+        <x:v>Next sign-in</x:v>
+      </x:c>
+      <x:c r="H7" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A8" s="116" t="str">
+        <x:v>Viewer</x:v>
+      </x:c>
+      <x:c r="B8" s="113" t="str">
+        <x:v>Per assigned Project</x:v>
+      </x:c>
+      <x:c r="C8" s="113" t="str">
+        <x:v>No Team membership</x:v>
+      </x:c>
+      <x:c r="D8" s="113" t="str">
+        <x:v>Read-only Project content</x:v>
+      </x:c>
+      <x:c r="E8" s="113" t="str">
+        <x:v>No structural administration</x:v>
+      </x:c>
+      <x:c r="F8" s="113" t="str">
+        <x:v>Assigned Project only</x:v>
+      </x:c>
+      <x:c r="G8" s="113" t="str">
+        <x:v>Next sign-in</x:v>
+      </x:c>
+      <x:c r="H8" s="119" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
+      <x:c r="A9" s="117" t="str">
+        <x:v>No Access</x:v>
+      </x:c>
+      <x:c r="B9" s="114" t="str">
+        <x:v>Default for every unassigned Project</x:v>
+      </x:c>
+      <x:c r="C9" s="114" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="D9" s="114" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E9" s="114" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="F9" s="114" t="str">
+        <x:v>Hidden; direct URL denied or safely not found</x:v>
+      </x:c>
+      <x:c r="G9" s="114" t="str">
+        <x:v>Next sign-in</x:v>
+      </x:c>
+      <x:c r="H9" s="120" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10"/>
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
+      <x:c r="A11" s="95" t="str">
+        <x:v>Required Access Re-test Scenarios</x:v>
+      </x:c>
+      <x:c r="B11" s="95"/>
+      <x:c r="C11" s="95"/>
+      <x:c r="D11" s="95"/>
+      <x:c r="E11" s="95"/>
+      <x:c r="F11" s="95"/>
+      <x:c r="G11" s="95"/>
+      <x:c r="H11" s="95"/>
+    </x:row>
+    <x:row r="12" ht="30" hidden="0" customHeight="1">
+      <x:c r="A12" s="104" t="str">
+        <x:v>Scenario ID</x:v>
+      </x:c>
+      <x:c r="B12" s="104" t="str">
+        <x:v>Business Rule</x:v>
+      </x:c>
+      <x:c r="C12" s="104" t="str">
+        <x:v>Precondition</x:v>
+      </x:c>
+      <x:c r="D12" s="104" t="str">
+        <x:v>Action</x:v>
+      </x:c>
+      <x:c r="E12" s="104" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="F12" s="104" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="G12" s="104" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="H12" s="104" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A13" s="115" t="str">
+        <x:v>P4-RBAC-001</x:v>
+      </x:c>
+      <x:c r="B13" s="112" t="str">
+        <x:v>Permission Model is read-only</x:v>
+      </x:c>
+      <x:c r="C13" s="112" t="str">
+        <x:v>Sign in as WA</x:v>
+      </x:c>
+      <x:c r="D13" s="112" t="str">
+        <x:v>Open Settings &gt; Permission Model</x:v>
+      </x:c>
+      <x:c r="E13" s="112" t="str">
+        <x:v>Capability reference is visible; no editable permission matrix</x:v>
+      </x:c>
+      <x:c r="F13" s="112" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G13" s="112" t="str"/>
+      <x:c r="H13" s="112" t="str"/>
+    </x:row>
+    <x:row r="14" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A14" s="116" t="str">
+        <x:v>P4-RBAC-002</x:v>
+      </x:c>
+      <x:c r="B14" s="113" t="str">
+        <x:v>WA is company-level only</x:v>
+      </x:c>
+      <x:c r="C14" s="113" t="str">
+        <x:v>WA account exists</x:v>
+      </x:c>
+      <x:c r="D14" s="113" t="str">
+        <x:v>Open Users and Project Users &amp; Permissions</x:v>
+      </x:c>
+      <x:c r="E14" s="113" t="str">
+        <x:v>WA detail is read-only and WA is excluded from Project member lists</x:v>
+      </x:c>
+      <x:c r="F14" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G14" s="113" t="str"/>
+      <x:c r="H14" s="113" t="str"/>
+    </x:row>
+    <x:row r="15" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A15" s="116" t="str">
+        <x:v>P4-RBAC-003</x:v>
+      </x:c>
+      <x:c r="B15" s="113" t="str">
+        <x:v>Project access is independent</x:v>
+      </x:c>
+      <x:c r="C15" s="113" t="str">
+        <x:v>User has Admin in Project A only</x:v>
+      </x:c>
+      <x:c r="D15" s="113" t="str">
+        <x:v>Open Project B</x:v>
+      </x:c>
+      <x:c r="E15" s="113" t="str">
+        <x:v>Project B remains No Access until WA explicitly assigns access</x:v>
+      </x:c>
+      <x:c r="F15" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G15" s="113" t="str"/>
+      <x:c r="H15" s="113" t="str"/>
+    </x:row>
+    <x:row r="16" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A16" s="116" t="str">
+        <x:v>P4-RBAC-004</x:v>
+      </x:c>
+      <x:c r="B16" s="113" t="str">
+        <x:v>Admin covers all Teams</x:v>
+      </x:c>
+      <x:c r="C16" s="113" t="str">
+        <x:v>User has Admin in Project A</x:v>
+      </x:c>
+      <x:c r="D16" s="113" t="str">
+        <x:v>Open Project A and Team-scoped delivery screens</x:v>
+      </x:c>
+      <x:c r="E16" s="113" t="str">
+        <x:v>All Teams and delivery administration are available</x:v>
+      </x:c>
+      <x:c r="F16" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G16" s="113" t="str"/>
+      <x:c r="H16" s="113" t="str"/>
+    </x:row>
+    <x:row r="17" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A17" s="116" t="str">
+        <x:v>P4-RBAC-005</x:v>
+      </x:c>
+      <x:c r="B17" s="113" t="str">
+        <x:v>Admin cannot change structure</x:v>
+      </x:c>
+      <x:c r="C17" s="113" t="str">
+        <x:v>User has Admin in Project A</x:v>
+      </x:c>
+      <x:c r="D17" s="113" t="str">
+        <x:v>Open Settings &gt; Workspaces &amp; Projects</x:v>
+      </x:c>
+      <x:c r="E17" s="113" t="str">
+        <x:v>Project Details, Teams, and Users &amp; Permissions are read-only</x:v>
+      </x:c>
+      <x:c r="F17" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G17" s="113" t="str"/>
+      <x:c r="H17" s="113" t="str"/>
+    </x:row>
+    <x:row r="18" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A18" s="116" t="str">
+        <x:v>P4-RBAC-006</x:v>
+      </x:c>
+      <x:c r="B18" s="113" t="str">
+        <x:v>Editor is Team-scoped</x:v>
+      </x:c>
+      <x:c r="C18" s="113" t="str">
+        <x:v>User has Editor in Project A / Team 1</x:v>
+      </x:c>
+      <x:c r="D18" s="113" t="str">
+        <x:v>Open backlog, quality, and iteration status</x:v>
+      </x:c>
+      <x:c r="E18" s="113" t="str">
+        <x:v>CRUD delivery items only in Team 1; no admin/report surfaces</x:v>
+      </x:c>
+      <x:c r="F18" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G18" s="113" t="str"/>
+      <x:c r="H18" s="113" t="str"/>
+    </x:row>
+    <x:row r="19" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A19" s="116" t="str">
+        <x:v>P4-RBAC-007</x:v>
+      </x:c>
+      <x:c r="B19" s="113" t="str">
+        <x:v>Viewer is Project read-only</x:v>
+      </x:c>
+      <x:c r="C19" s="113" t="str">
+        <x:v>User has Viewer in Project A</x:v>
+      </x:c>
+      <x:c r="D19" s="113" t="str">
+        <x:v>Open Project A screens</x:v>
+      </x:c>
+      <x:c r="E19" s="113" t="str">
+        <x:v>Content is visible and all mutations are unavailable</x:v>
+      </x:c>
+      <x:c r="F19" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G19" s="113" t="str"/>
+      <x:c r="H19" s="113" t="str"/>
+    </x:row>
+    <x:row r="20" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A20" s="116" t="str">
+        <x:v>P4-RBAC-008</x:v>
+      </x:c>
+      <x:c r="B20" s="113" t="str">
+        <x:v>No Access is hidden and denied</x:v>
+      </x:c>
+      <x:c r="C20" s="113" t="str">
+        <x:v>User has No Access in Project B</x:v>
+      </x:c>
+      <x:c r="D20" s="113" t="str">
+        <x:v>Use selector and direct URL</x:v>
+      </x:c>
+      <x:c r="E20" s="113" t="str">
+        <x:v>Project B is absent and direct navigation is safely denied</x:v>
+      </x:c>
+      <x:c r="F20" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G20" s="113" t="str"/>
+      <x:c r="H20" s="113" t="str"/>
+    </x:row>
+    <x:row r="21" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A21" s="116" t="str">
+        <x:v>P4-RBAC-009</x:v>
+      </x:c>
+      <x:c r="B21" s="113" t="str">
+        <x:v>User-first and Project-first journeys stay synchronized</x:v>
+      </x:c>
+      <x:c r="C21" s="113" t="str">
+        <x:v>Sign in as WA</x:v>
+      </x:c>
+      <x:c r="D21" s="113" t="str">
+        <x:v>Assign/change/remove Project access from either journey</x:v>
+      </x:c>
+      <x:c r="E21" s="113" t="str">
+        <x:v>Both journeys show the same Access Level and membership state</x:v>
+      </x:c>
+      <x:c r="F21" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G21" s="113" t="str"/>
+      <x:c r="H21" s="113" t="str"/>
+    </x:row>
+    <x:row r="22" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A22" s="116" t="str">
+        <x:v>P4-RBAC-010</x:v>
+      </x:c>
+      <x:c r="B22" s="113" t="str">
+        <x:v>Team setup can assign access</x:v>
+      </x:c>
+      <x:c r="C22" s="113" t="str">
+        <x:v>Sign in as WA</x:v>
+      </x:c>
+      <x:c r="D22" s="113" t="str">
+        <x:v>Create/edit Team and add existing user</x:v>
+      </x:c>
+      <x:c r="E22" s="113" t="str">
+        <x:v>Admin becomes All Teams; Editor joins the selected Team</x:v>
+      </x:c>
+      <x:c r="F22" s="113" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G22" s="113" t="str"/>
+      <x:c r="H22" s="113" t="str"/>
+    </x:row>
+    <x:row r="23" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A23" s="117" t="str">
+        <x:v>P4-RBAC-011</x:v>
+      </x:c>
+      <x:c r="B23" s="114" t="str">
+        <x:v>Notification route rechecks access</x:v>
+      </x:c>
+      <x:c r="C23" s="114" t="str">
+        <x:v>Assignment or Note mention notification exists</x:v>
+      </x:c>
+      <x:c r="D23" s="114" t="str">
+        <x:v>Click notification after access changes</x:v>
+      </x:c>
+      <x:c r="E23" s="114" t="str">
+        <x:v>User reaches the related Work Item only when current access allows it</x:v>
+      </x:c>
+      <x:c r="F23" s="114" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="G23" s="114" t="str"/>
+      <x:c r="H23" s="114" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A11:H11"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="F13:F23">
+      <x:formula1>"Not Run,Pass,Fail,Blocked"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>